<commit_message>
update with logo officiel
</commit_message>
<xml_diff>
--- a/MyModels_V2/Cartes.xlsx
+++ b/MyModels_V2/Cartes.xlsx
@@ -48,34 +48,34 @@
     <t>Photo</t>
   </si>
   <si>
-    <t>102060000001R</t>
-  </si>
-  <si>
-    <t>8509464113</t>
-  </si>
-  <si>
-    <t>ZOUNGRANA</t>
-  </si>
-  <si>
-    <t>B Odilon Isaïe</t>
-  </si>
-  <si>
-    <t>20/01/1992</t>
-  </si>
-  <si>
-    <t>Sapone</t>
-  </si>
-  <si>
-    <t>10/06/2024</t>
-  </si>
-  <si>
-    <t>ZOUNGRANA Fleurty (+226) 63641254</t>
-  </si>
-  <si>
-    <t>http://localhost:8089/api/affiliation-immatriculation/xyz/7369676e61747572652d6361727465</t>
-  </si>
-  <si>
-    <t>http://localhost:8089/api/affiliation-immatriculation/export/photo/87.jpg</t>
+    <t>111010000002G</t>
+  </si>
+  <si>
+    <t>0509081851</t>
+  </si>
+  <si>
+    <t>KOUGOUINDIGA</t>
+  </si>
+  <si>
+    <t>SENI</t>
+  </si>
+  <si>
+    <t>31/12/1981</t>
+  </si>
+  <si>
+    <t>Niongnongo</t>
+  </si>
+  <si>
+    <t>27/05/2025</t>
+  </si>
+  <si>
+    <t>KOUGOUINDIGA IBRAHIM (+226) 78218356</t>
+  </si>
+  <si>
+    <t>http://sigramu.cnamu.bf/api/affiliation-immatriculation/xyz/7369676e61747572652d6361727465</t>
+  </si>
+  <si>
+    <t>http://sigramu.cnamu.bf/api/affiliation-immatriculation/export/photo/1566.jpg</t>
   </si>
 </sst>
 </file>

</xml_diff>